<commit_message>
Added frequency statistic for CCs; fixed bugs with data that contained outdated CC keywords
</commit_message>
<xml_diff>
--- a/MRCC_Updated.xlsx
+++ b/MRCC_Updated.xlsx
@@ -434,7 +434,7 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>If Y, Which CC?</t>
+          <t>If Y, Which CC (Passive)?</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
@@ -444,7 +444,7 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>If Y, Which CC?.1</t>
+          <t>If Y, Which CC (Melee)?</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
@@ -459,7 +459,7 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>If Y, Which CC?.2</t>
+          <t>If Y, Which CC (Primary)?</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
@@ -474,7 +474,7 @@
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>If Y, Which CC?.3</t>
+          <t>If Y, Which CC (Secondary)?</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
@@ -489,7 +489,7 @@
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>If Y, What CC?</t>
+          <t>If Y, Which CC (A1)?</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
@@ -504,7 +504,7 @@
       </c>
       <c r="S1" t="inlineStr">
         <is>
-          <t>If Y, What CC?.1</t>
+          <t>If Y, Which CC (A2)?</t>
         </is>
       </c>
       <c r="T1" t="inlineStr">
@@ -519,7 +519,7 @@
       </c>
       <c r="V1" t="inlineStr">
         <is>
-          <t>If Y, What CC?.2</t>
+          <t>If Y, Which CC (A3)?</t>
         </is>
       </c>
       <c r="W1" t="inlineStr">
@@ -534,7 +534,7 @@
       </c>
       <c r="Y1" t="inlineStr">
         <is>
-          <t>If Y, What CC?.3</t>
+          <t>If Y, Which CC (A4)?</t>
         </is>
       </c>
       <c r="Z1" t="inlineStr">
@@ -549,7 +549,7 @@
       </c>
       <c r="AB1" t="inlineStr">
         <is>
-          <t>If Y, What CC?.4</t>
+          <t>If Y, Which CC (Ult)?</t>
         </is>
       </c>
       <c r="AC1" t="inlineStr">
@@ -1254,7 +1254,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Displacement</t>
+          <t>Launched</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1603,7 +1603,7 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>Knocked Pulled</t>
+          <t>Pulled</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">

</xml_diff>